<commit_message>
Drop MAPE from the 10_11 comparison table.
The 10_11 notebook reports R², MAE, MSE, and RMSE only.

Co-authored-by: thewrongcoder <thewrongcoder@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/results/10_11_comparison_400k_train_100k_test.xlsx
+++ b/results/10_11_comparison_400k_train_100k_test.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -442,11 +442,6 @@
           <t>RMSE</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>MAPE (%)</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -466,9 +461,6 @@
       <c r="E2" t="n">
         <v>0.7463</v>
       </c>
-      <c r="F2" t="n">
-        <v>123.3653</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -488,9 +480,6 @@
       <c r="E3" t="n">
         <v>0.6913</v>
       </c>
-      <c r="F3" t="n">
-        <v>160.0843</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -510,9 +499,6 @@
       <c r="E4" t="n">
         <v>0.7027</v>
       </c>
-      <c r="F4" t="n">
-        <v>151.7027</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -532,9 +518,6 @@
       <c r="E5" t="n">
         <v>0.6937</v>
       </c>
-      <c r="F5" t="n">
-        <v>154.8249</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -554,9 +537,6 @@
       <c r="E6" t="n">
         <v>0.6891</v>
       </c>
-      <c r="F6" t="n">
-        <v>167.1634</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -576,9 +556,6 @@
       <c r="E7" t="n">
         <v>0.6848</v>
       </c>
-      <c r="F7" t="n">
-        <v>164.5762</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -598,9 +575,6 @@
       <c r="E8" t="n">
         <v>0.6846</v>
       </c>
-      <c r="F8" t="n">
-        <v>164.9302</v>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -619,9 +593,6 @@
       </c>
       <c r="E9" t="n">
         <v>1.3783</v>
-      </c>
-      <c r="F9" t="n">
-        <v>115.7349</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Re-score TabPFN with 64-row CPU batches and record the updated table.
Pooled TabPFN R² is 0.0113 (no longer negative). Other models are unchanged on the same 400k/100k split.

Co-authored-by: thewrongcoder <thewrongcoder@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/results/10_11_comparison_400k_train_100k_test.xlsx
+++ b/results/10_11_comparison_400k_train_100k_test.xlsx
@@ -583,16 +583,16 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-2.1222</v>
+        <v>0.0113</v>
       </c>
       <c r="C9" t="n">
-        <v>0.1762</v>
+        <v>0.1219</v>
       </c>
       <c r="D9" t="n">
-        <v>1.8997</v>
+        <v>0.6016</v>
       </c>
       <c r="E9" t="n">
-        <v>1.3783</v>
+        <v>0.7756</v>
       </c>
     </row>
   </sheetData>

</xml_diff>